<commit_message>
Revert "new new upright"
This reverts commit 7e3219d21d8910d8b06cb5887a73d4343031a4d0.
</commit_message>
<xml_diff>
--- a/Suspension/Final Suspension Parts/3D_Suspension_Analyzer/3D_Suspension_Analyzer_V2.xlsx
+++ b/Suspension/Final Suspension Parts/3D_Suspension_Analyzer/3D_Suspension_Analyzer_V2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\share\OneDrive\Documents\Personal Projects\GOGO Kart\CAD\GOGO_KART_FSAE\Suspension\Final Suspension Parts\3D_Suspension_Analyzer\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\share\OneDrive\Documents\Personal Projects\GOGO Kart\CAD\GOGO_KART_FSAE\Suspension\3D_Suspension_Analyzer\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A13BAED-1AD7-49F6-B4DF-75C98441FBE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A02D5118-3614-407C-A7E4-6E873F1678A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Suspension Analyzer" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="625" uniqueCount="348">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="622" uniqueCount="347">
   <si>
     <t>Camber offset (deg):</t>
   </si>
@@ -945,6 +945,12 @@
     <t>Pedal Ratio (PR)</t>
   </si>
   <si>
+    <t>Supplied Front Braking Torque</t>
+  </si>
+  <si>
+    <t>Supplied Rear Braking Torque</t>
+  </si>
+  <si>
     <t>Front Caliper Piston Area</t>
   </si>
   <si>
@@ -1008,6 +1014,9 @@
     <t>psi</t>
   </si>
   <si>
+    <t>500-700</t>
+  </si>
+  <si>
     <t>Outboard Suspension Bearing Housing Sizing</t>
   </si>
   <si>
@@ -1069,18 +1078,6 @@
   </si>
   <si>
     <t>(Kingpin inclination) front view angle between the steering axis and vertical</t>
-  </si>
-  <si>
-    <t>Required Front Braking Torque (per wheel)</t>
-  </si>
-  <si>
-    <t>Required Rear Braking Torque (per wheel)</t>
-  </si>
-  <si>
-    <t>Supplied Front Braking Torque (per wheel)</t>
-  </si>
-  <si>
-    <t>Supplied Rear Braking Torque (per wheel)</t>
   </si>
 </sst>
 </file>
@@ -1301,7 +1298,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1380,8 +1377,23 @@
     <xf numFmtId="1" fontId="4" fillId="16" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1424,40 +1436,14 @@
     <xf numFmtId="0" fontId="0" fillId="16" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="16" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3010,69 +2996,69 @@
       </c>
     </row>
     <row r="3" spans="3:61" x14ac:dyDescent="0.25">
-      <c r="C3" s="56" t="s">
+      <c r="C3" s="40" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="49"/>
-      <c r="E3" s="49"/>
-      <c r="F3" s="50"/>
-      <c r="H3" s="56" t="s">
+      <c r="D3" s="33"/>
+      <c r="E3" s="33"/>
+      <c r="F3" s="34"/>
+      <c r="H3" s="40" t="s">
         <v>2</v>
       </c>
-      <c r="I3" s="49"/>
-      <c r="J3" s="49"/>
-      <c r="K3" s="50"/>
-      <c r="M3" s="48" t="s">
+      <c r="I3" s="33"/>
+      <c r="J3" s="33"/>
+      <c r="K3" s="34"/>
+      <c r="M3" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="N3" s="49"/>
-      <c r="O3" s="49"/>
-      <c r="P3" s="49"/>
-      <c r="Q3" s="50"/>
-      <c r="T3" s="51" t="s">
+      <c r="N3" s="33"/>
+      <c r="O3" s="33"/>
+      <c r="P3" s="33"/>
+      <c r="Q3" s="34"/>
+      <c r="T3" s="35" t="s">
         <v>216</v>
       </c>
-      <c r="U3" s="52"/>
-      <c r="V3" s="52"/>
-      <c r="W3" s="52"/>
-      <c r="X3" s="52"/>
-      <c r="Y3" s="52"/>
-      <c r="Z3" s="52"/>
-      <c r="AA3" s="52"/>
-      <c r="AB3" s="52"/>
-      <c r="AC3" s="52"/>
-      <c r="AD3" s="52"/>
-      <c r="AE3" s="52"/>
-      <c r="AF3" s="52"/>
-      <c r="AG3" s="52"/>
-      <c r="AH3" s="52"/>
-      <c r="AI3" s="52"/>
-      <c r="AJ3" s="52"/>
-      <c r="AK3" s="52"/>
-      <c r="AL3" s="52"/>
-      <c r="AM3" s="52"/>
-      <c r="AN3" s="52"/>
-      <c r="AO3" s="52"/>
-      <c r="AP3" s="52"/>
-      <c r="AQ3" s="52"/>
-      <c r="AR3" s="52"/>
-      <c r="AS3" s="52"/>
-      <c r="AT3" s="52"/>
-      <c r="AU3" s="52"/>
-      <c r="AV3" s="52"/>
-      <c r="AW3" s="52"/>
-      <c r="AX3" s="52"/>
-      <c r="AY3" s="52"/>
-      <c r="AZ3" s="52"/>
-      <c r="BA3" s="52"/>
-      <c r="BB3" s="52"/>
-      <c r="BC3" s="52"/>
-      <c r="BD3" s="52"/>
-      <c r="BE3" s="52"/>
-      <c r="BF3" s="52"/>
-      <c r="BG3" s="52"/>
-      <c r="BH3" s="52"/>
-      <c r="BI3" s="52"/>
+      <c r="U3" s="36"/>
+      <c r="V3" s="36"/>
+      <c r="W3" s="36"/>
+      <c r="X3" s="36"/>
+      <c r="Y3" s="36"/>
+      <c r="Z3" s="36"/>
+      <c r="AA3" s="36"/>
+      <c r="AB3" s="36"/>
+      <c r="AC3" s="36"/>
+      <c r="AD3" s="36"/>
+      <c r="AE3" s="36"/>
+      <c r="AF3" s="36"/>
+      <c r="AG3" s="36"/>
+      <c r="AH3" s="36"/>
+      <c r="AI3" s="36"/>
+      <c r="AJ3" s="36"/>
+      <c r="AK3" s="36"/>
+      <c r="AL3" s="36"/>
+      <c r="AM3" s="36"/>
+      <c r="AN3" s="36"/>
+      <c r="AO3" s="36"/>
+      <c r="AP3" s="36"/>
+      <c r="AQ3" s="36"/>
+      <c r="AR3" s="36"/>
+      <c r="AS3" s="36"/>
+      <c r="AT3" s="36"/>
+      <c r="AU3" s="36"/>
+      <c r="AV3" s="36"/>
+      <c r="AW3" s="36"/>
+      <c r="AX3" s="36"/>
+      <c r="AY3" s="36"/>
+      <c r="AZ3" s="36"/>
+      <c r="BA3" s="36"/>
+      <c r="BB3" s="36"/>
+      <c r="BC3" s="36"/>
+      <c r="BD3" s="36"/>
+      <c r="BE3" s="36"/>
+      <c r="BF3" s="36"/>
+      <c r="BG3" s="36"/>
+      <c r="BH3" s="36"/>
+      <c r="BI3" s="36"/>
     </row>
     <row r="4" spans="3:61" x14ac:dyDescent="0.25">
       <c r="C4" s="2" t="s">
@@ -4887,13 +4873,13 @@
       <c r="F13" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="M13" s="48" t="s">
+      <c r="M13" s="32" t="s">
         <v>99</v>
       </c>
-      <c r="N13" s="49"/>
-      <c r="O13" s="49"/>
-      <c r="P13" s="49"/>
-      <c r="Q13" s="50"/>
+      <c r="N13" s="33"/>
+      <c r="O13" s="33"/>
+      <c r="P13" s="33"/>
+      <c r="Q13" s="34"/>
       <c r="T13" s="22">
         <v>-12</v>
       </c>
@@ -5075,19 +5061,19 @@
       <c r="F14" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="H14" s="48" t="s">
+      <c r="H14" s="32" t="s">
         <v>102</v>
       </c>
-      <c r="I14" s="49"/>
-      <c r="J14" s="49"/>
-      <c r="K14" s="50"/>
-      <c r="M14" s="55">
-        <v>0</v>
-      </c>
-      <c r="N14" s="49"/>
-      <c r="O14" s="49"/>
-      <c r="P14" s="49"/>
-      <c r="Q14" s="50"/>
+      <c r="I14" s="33"/>
+      <c r="J14" s="33"/>
+      <c r="K14" s="34"/>
+      <c r="M14" s="39">
+        <v>0</v>
+      </c>
+      <c r="N14" s="33"/>
+      <c r="O14" s="33"/>
+      <c r="P14" s="33"/>
+      <c r="Q14" s="34"/>
       <c r="T14" s="22">
         <v>-11</v>
       </c>
@@ -5825,12 +5811,12 @@
       </c>
     </row>
     <row r="18" spans="3:61" x14ac:dyDescent="0.25">
-      <c r="C18" s="48" t="s">
+      <c r="C18" s="32" t="s">
         <v>111</v>
       </c>
-      <c r="D18" s="49"/>
-      <c r="E18" s="49"/>
-      <c r="F18" s="50"/>
+      <c r="D18" s="33"/>
+      <c r="E18" s="33"/>
+      <c r="F18" s="34"/>
       <c r="H18" s="5" t="s">
         <v>112</v>
       </c>
@@ -7377,12 +7363,12 @@
       <c r="F26" s="3" t="s">
         <v>138</v>
       </c>
-      <c r="H26" s="56" t="s">
+      <c r="H26" s="40" t="s">
         <v>139</v>
       </c>
-      <c r="I26" s="49"/>
-      <c r="J26" s="49"/>
-      <c r="K26" s="50"/>
+      <c r="I26" s="33"/>
+      <c r="J26" s="33"/>
+      <c r="K26" s="34"/>
       <c r="T26" s="22">
         <v>1</v>
       </c>
@@ -9682,12 +9668,12 @@
       </c>
     </row>
     <row r="38" spans="3:61" x14ac:dyDescent="0.25">
-      <c r="C38" s="53" t="s">
+      <c r="C38" s="37" t="s">
         <v>169</v>
       </c>
-      <c r="D38" s="54"/>
-      <c r="E38" s="54"/>
-      <c r="F38" s="54"/>
+      <c r="D38" s="38"/>
+      <c r="E38" s="38"/>
+      <c r="F38" s="38"/>
       <c r="H38" s="4" t="s">
         <v>27</v>
       </c>
@@ -10270,7 +10256,7 @@
         <v>89</v>
       </c>
       <c r="F41" s="6" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="H41" s="4" t="s">
         <v>177</v>
@@ -11371,12 +11357,12 @@
       </c>
     </row>
     <row r="57" spans="8:11" x14ac:dyDescent="0.25">
-      <c r="H57" s="48" t="s">
+      <c r="H57" s="32" t="s">
         <v>204</v>
       </c>
-      <c r="I57" s="49"/>
-      <c r="J57" s="49"/>
-      <c r="K57" s="50"/>
+      <c r="I57" s="33"/>
+      <c r="J57" s="33"/>
+      <c r="K57" s="34"/>
     </row>
     <row r="58" spans="8:11" x14ac:dyDescent="0.25">
       <c r="H58" s="2" t="s">
@@ -11569,18 +11555,18 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B2" s="57" t="s">
-        <v>323</v>
-      </c>
-      <c r="C2" s="57"/>
-      <c r="D2" s="57"/>
+      <c r="B2" s="55" t="s">
+        <v>326</v>
+      </c>
+      <c r="C2" s="55"/>
+      <c r="D2" s="55"/>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B3" s="58" t="s">
+      <c r="B3" s="57" t="s">
         <v>223</v>
       </c>
-      <c r="C3" s="58"/>
-      <c r="D3" s="58"/>
+      <c r="C3" s="57"/>
+      <c r="D3" s="57"/>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B4" s="17" t="s">
@@ -11589,97 +11575,97 @@
       <c r="C4" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="32" t="s">
+      <c r="D4" s="56" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B5" s="32" t="s">
+      <c r="B5" s="56" t="s">
+        <v>331</v>
+      </c>
+      <c r="C5" s="56">
+        <v>12</v>
+      </c>
+      <c r="D5" s="56" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="6" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B6" s="56" t="s">
+        <v>243</v>
+      </c>
+      <c r="C6" s="56">
+        <v>1.169</v>
+      </c>
+      <c r="D6" s="56" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="7" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B7" s="56" t="s">
+        <v>290</v>
+      </c>
+      <c r="C7" s="56">
+        <v>323</v>
+      </c>
+      <c r="D7" s="56" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="8" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B8" s="56" t="s">
+        <v>327</v>
+      </c>
+      <c r="C8" s="56">
+        <v>1.5</v>
+      </c>
+      <c r="D8" s="56" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="9" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B9" s="56" t="s">
         <v>328</v>
       </c>
-      <c r="C5" s="32">
-        <v>12</v>
-      </c>
-      <c r="D5" s="32" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="6" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B6" s="32" t="s">
-        <v>243</v>
-      </c>
-      <c r="C6" s="32">
-        <v>1.169</v>
-      </c>
-      <c r="D6" s="32" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="7" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B7" s="32" t="s">
-        <v>290</v>
-      </c>
-      <c r="C7" s="32">
-        <v>323</v>
-      </c>
-      <c r="D7" s="32" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="8" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B8" s="32" t="s">
-        <v>324</v>
-      </c>
-      <c r="C8" s="32">
-        <v>1.5</v>
-      </c>
-      <c r="D8" s="32" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="9" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B9" s="32" t="s">
-        <v>325</v>
-      </c>
-      <c r="C9" s="32">
+      <c r="C9" s="56">
         <v>25</v>
       </c>
-      <c r="D9" s="32" t="s">
+      <c r="D9" s="56" t="s">
         <v>233</v>
       </c>
     </row>
     <row r="10" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B10" s="58" t="s">
+      <c r="B10" s="57" t="s">
         <v>249</v>
       </c>
-      <c r="C10" s="58"/>
-      <c r="D10" s="58"/>
+      <c r="C10" s="57"/>
+      <c r="D10" s="57"/>
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B11" s="32" t="s">
-        <v>326</v>
-      </c>
-      <c r="C11" s="32">
+      <c r="B11" s="56" t="s">
+        <v>329</v>
+      </c>
+      <c r="C11" s="56">
         <f>(C7*9.8*C8*(C9/100))/((C5/1000)*(C6/1000)*(2))/(10^6)</f>
         <v>42.309131736526943</v>
       </c>
-      <c r="D11" s="32" t="s">
-        <v>327</v>
+      <c r="D11" s="56" t="s">
+        <v>330</v>
       </c>
     </row>
     <row r="14" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B14" s="57" t="s">
-        <v>329</v>
-      </c>
-      <c r="C14" s="57"/>
-      <c r="D14" s="57"/>
+      <c r="B14" s="55" t="s">
+        <v>332</v>
+      </c>
+      <c r="C14" s="55"/>
+      <c r="D14" s="55"/>
     </row>
     <row r="15" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B15" s="58" t="s">
+      <c r="B15" s="57" t="s">
         <v>223</v>
       </c>
-      <c r="C15" s="58"/>
-      <c r="D15" s="58"/>
+      <c r="C15" s="57"/>
+      <c r="D15" s="57"/>
     </row>
     <row r="16" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B16" s="17" t="s">
@@ -11688,75 +11674,75 @@
       <c r="C16" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="D16" s="32" t="s">
+      <c r="D16" s="56" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B17" s="32" t="s">
+      <c r="B17" s="56" t="s">
         <v>242</v>
       </c>
-      <c r="C17" s="32">
+      <c r="C17" s="56">
         <v>12</v>
       </c>
-      <c r="D17" s="32" t="s">
+      <c r="D17" s="56" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="18" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B18" s="32" t="s">
-        <v>330</v>
-      </c>
-      <c r="C18" s="32">
+      <c r="B18" s="56" t="s">
+        <v>333</v>
+      </c>
+      <c r="C18" s="56">
         <v>85</v>
       </c>
-      <c r="D18" s="32" t="s">
+      <c r="D18" s="56" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="19" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B19" s="32" t="s">
+      <c r="B19" s="56" t="s">
         <v>290</v>
       </c>
-      <c r="C19" s="32">
+      <c r="C19" s="56">
         <v>323</v>
       </c>
-      <c r="D19" s="32" t="s">
+      <c r="D19" s="56" t="s">
         <v>227</v>
       </c>
     </row>
     <row r="20" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B20" s="32" t="s">
-        <v>331</v>
-      </c>
-      <c r="C20" s="32">
+      <c r="B20" s="56" t="s">
+        <v>334</v>
+      </c>
+      <c r="C20" s="56">
         <v>1.5</v>
       </c>
-      <c r="D20" s="32" t="s">
+      <c r="D20" s="56" t="s">
         <v>221</v>
       </c>
     </row>
     <row r="21" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B21" s="32" t="s">
-        <v>325</v>
-      </c>
-      <c r="C21" s="32">
+      <c r="B21" s="56" t="s">
+        <v>328</v>
+      </c>
+      <c r="C21" s="56">
         <v>30</v>
       </c>
-      <c r="D21" s="32" t="s">
+      <c r="D21" s="56" t="s">
         <v>233</v>
       </c>
     </row>
     <row r="22" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B22" s="58" t="s">
+      <c r="B22" s="57" t="s">
         <v>249</v>
       </c>
-      <c r="C22" s="58"/>
-      <c r="D22" s="58"/>
+      <c r="C22" s="57"/>
+      <c r="D22" s="57"/>
     </row>
     <row r="23" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B23" s="5" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="C23" s="5">
         <f>(C19)*9.8*(C20)</f>
@@ -11768,7 +11754,7 @@
     </row>
     <row r="24" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B24" s="5" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="C24" s="30">
         <f>C23-C37</f>
@@ -11778,41 +11764,41 @@
     </row>
     <row r="25" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B25" s="5" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="C25" s="5">
         <f>(PI()*(C17/1000)^4) / 64</f>
         <v>1.0178760197630931E-9</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
     </row>
     <row r="26" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B26" s="32" t="s">
-        <v>326</v>
-      </c>
-      <c r="C26" s="32">
+      <c r="B26" s="56" t="s">
+        <v>329</v>
+      </c>
+      <c r="C26" s="56">
         <f>((C24*(C21/100))*(C18/1000)*(C17/2000)/C25)/10^6</f>
         <v>0.54923645172942581</v>
       </c>
-      <c r="D26" s="32" t="s">
-        <v>327</v>
+      <c r="D26" s="56" t="s">
+        <v>330</v>
       </c>
     </row>
     <row r="28" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B28" s="57" t="s">
-        <v>334</v>
-      </c>
-      <c r="C28" s="57"/>
-      <c r="D28" s="57"/>
+      <c r="B28" s="55" t="s">
+        <v>337</v>
+      </c>
+      <c r="C28" s="55"/>
+      <c r="D28" s="55"/>
     </row>
     <row r="29" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B29" s="58" t="s">
+      <c r="B29" s="57" t="s">
         <v>223</v>
       </c>
-      <c r="C29" s="58"/>
-      <c r="D29" s="58"/>
+      <c r="C29" s="57"/>
+      <c r="D29" s="57"/>
     </row>
     <row r="30" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B30" s="17" t="s">
@@ -11821,76 +11807,76 @@
       <c r="C30" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="D30" s="32" t="s">
+      <c r="D30" s="56" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="31" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B31" s="32" t="s">
+      <c r="B31" s="56" t="s">
+        <v>338</v>
+      </c>
+      <c r="C31" s="56">
+        <v>1.85</v>
+      </c>
+      <c r="D31" s="56" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="32" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B32" s="56" t="s">
+        <v>339</v>
+      </c>
+      <c r="C32" s="56">
+        <v>210</v>
+      </c>
+      <c r="D32" s="56" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="33" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B33" s="56" t="s">
+        <v>343</v>
+      </c>
+      <c r="C33" s="56">
+        <v>12</v>
+      </c>
+      <c r="D33" s="56" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="34" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B34" s="56" t="s">
+        <v>340</v>
+      </c>
+      <c r="C34" s="56">
+        <v>63</v>
+      </c>
+      <c r="D34" s="56" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="35" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B35" s="55" t="s">
+        <v>249</v>
+      </c>
+      <c r="C35" s="55"/>
+      <c r="D35" s="55"/>
+    </row>
+    <row r="36" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B36" s="58" t="s">
         <v>335</v>
       </c>
-      <c r="C31" s="32">
-        <v>1.85</v>
-      </c>
-      <c r="D31" s="32" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="32" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B32" s="32" t="s">
-        <v>336</v>
-      </c>
-      <c r="C32" s="32">
-        <v>210</v>
-      </c>
-      <c r="D32" s="32" t="s">
-        <v>339</v>
-      </c>
-    </row>
-    <row r="33" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B33" s="32" t="s">
-        <v>340</v>
-      </c>
-      <c r="C33" s="32">
-        <v>12</v>
-      </c>
-      <c r="D33" s="32" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="34" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B34" s="32" t="s">
-        <v>337</v>
-      </c>
-      <c r="C34" s="32">
-        <v>63</v>
-      </c>
-      <c r="D34" s="32" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="35" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B35" s="57" t="s">
-        <v>249</v>
-      </c>
-      <c r="C35" s="57"/>
-      <c r="D35" s="57"/>
-    </row>
-    <row r="36" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B36" s="33" t="s">
-        <v>332</v>
-      </c>
-      <c r="C36" s="33">
+      <c r="C36" s="58">
         <f>(PI()*(C33/1000)^4) / 64</f>
         <v>1.0178760197630931E-9</v>
       </c>
-      <c r="D36" s="33" t="s">
-        <v>333</v>
+      <c r="D36" s="58" t="s">
+        <v>336</v>
       </c>
     </row>
     <row r="37" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B37" s="33" t="s">
-        <v>338</v>
+      <c r="B37" s="58" t="s">
+        <v>341</v>
       </c>
       <c r="C37" s="5">
         <f>((C31/1000)*3*(C32*10^9)*(C36))/(C34/1000)^3</f>
@@ -11901,12 +11887,12 @@
       </c>
     </row>
     <row r="38" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B38" s="32"/>
-      <c r="C38" s="32">
+      <c r="B38" s="56"/>
+      <c r="C38" s="56">
         <f>C37/9.8</f>
         <v>484.12714778351665</v>
       </c>
-      <c r="D38" s="32"/>
+      <c r="D38" s="56"/>
     </row>
     <row r="39" spans="2:4" x14ac:dyDescent="0.25">
       <c r="C39">
@@ -11916,6 +11902,7 @@
     </row>
   </sheetData>
   <mergeCells count="9">
+    <mergeCell ref="B28:D28"/>
     <mergeCell ref="B29:D29"/>
     <mergeCell ref="B35:D35"/>
     <mergeCell ref="B15:D15"/>
@@ -11924,7 +11911,6 @@
     <mergeCell ref="B3:D3"/>
     <mergeCell ref="B10:D10"/>
     <mergeCell ref="B14:D14"/>
-    <mergeCell ref="B28:D28"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -11941,7 +11927,7 @@
     <col min="5" max="5" width="12.7109375" customWidth="1"/>
     <col min="6" max="6" width="8.42578125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="39.85546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="5.85546875" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="32.28515625" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="9.28515625" customWidth="1"/>
@@ -11949,24 +11935,24 @@
   </cols>
   <sheetData>
     <row r="3" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C3" s="38" t="s">
+      <c r="C3" s="45" t="s">
         <v>245</v>
       </c>
-      <c r="D3" s="38"/>
-      <c r="E3" s="38"/>
-      <c r="F3" s="38"/>
+      <c r="D3" s="45"/>
+      <c r="E3" s="45"/>
+      <c r="F3" s="45"/>
       <c r="G3" s="26"/>
-      <c r="I3" s="38" t="s">
+      <c r="I3" s="45" t="s">
         <v>290</v>
       </c>
-      <c r="J3" s="38"/>
-      <c r="K3" s="38"/>
+      <c r="J3" s="45"/>
+      <c r="K3" s="45"/>
     </row>
     <row r="4" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C4" s="46" t="s">
+      <c r="C4" s="53" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="46"/>
+      <c r="D4" s="53"/>
       <c r="E4" s="27" t="s">
         <v>5</v>
       </c>
@@ -11984,12 +11970,12 @@
       </c>
     </row>
     <row r="5" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C5" s="34" t="s">
+      <c r="C5" s="41" t="s">
         <v>223</v>
       </c>
-      <c r="D5" s="34"/>
-      <c r="E5" s="34"/>
-      <c r="F5" s="34"/>
+      <c r="D5" s="41"/>
+      <c r="E5" s="41"/>
+      <c r="F5" s="41"/>
       <c r="I5" s="5" t="s">
         <v>293</v>
       </c>
@@ -12002,10 +11988,10 @@
       </c>
     </row>
     <row r="6" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C6" s="47" t="s">
+      <c r="C6" s="54" t="s">
         <v>240</v>
       </c>
-      <c r="D6" s="47"/>
+      <c r="D6" s="54"/>
       <c r="E6" s="24">
         <v>0.28360000000000002</v>
       </c>
@@ -12024,10 +12010,10 @@
       </c>
     </row>
     <row r="7" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C7" s="47" t="s">
+      <c r="C7" s="54" t="s">
         <v>242</v>
       </c>
-      <c r="D7" s="47"/>
+      <c r="D7" s="54"/>
       <c r="E7" s="24">
         <v>1</v>
       </c>
@@ -12046,10 +12032,10 @@
       </c>
     </row>
     <row r="8" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C8" s="47" t="s">
+      <c r="C8" s="54" t="s">
         <v>243</v>
       </c>
-      <c r="D8" s="47"/>
+      <c r="D8" s="54"/>
       <c r="E8" s="24">
         <v>8.3000000000000004E-2</v>
       </c>
@@ -12068,10 +12054,10 @@
       </c>
     </row>
     <row r="9" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C9" s="47" t="s">
+      <c r="C9" s="54" t="s">
         <v>246</v>
       </c>
-      <c r="D9" s="47"/>
+      <c r="D9" s="54"/>
       <c r="E9" s="24">
         <v>157.21</v>
       </c>
@@ -12080,23 +12066,23 @@
       </c>
     </row>
     <row r="10" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C10" s="43" t="s">
+      <c r="C10" s="50" t="s">
         <v>249</v>
       </c>
-      <c r="D10" s="44"/>
-      <c r="E10" s="44"/>
-      <c r="F10" s="45"/>
-      <c r="I10" s="35" t="s">
+      <c r="D10" s="51"/>
+      <c r="E10" s="51"/>
+      <c r="F10" s="52"/>
+      <c r="I10" s="42" t="s">
         <v>222</v>
       </c>
-      <c r="J10" s="36"/>
-      <c r="K10" s="37"/>
+      <c r="J10" s="43"/>
+      <c r="K10" s="44"/>
     </row>
     <row r="11" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C11" s="47" t="s">
+      <c r="C11" s="54" t="s">
         <v>241</v>
       </c>
-      <c r="D11" s="47"/>
+      <c r="D11" s="54"/>
       <c r="E11" s="24">
         <f>(E7-2*E8)</f>
         <v>0.83399999999999996</v>
@@ -12115,10 +12101,10 @@
       </c>
     </row>
     <row r="12" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C12" s="47" t="s">
+      <c r="C12" s="54" t="s">
         <v>250</v>
       </c>
-      <c r="D12" s="47"/>
+      <c r="D12" s="54"/>
       <c r="E12" s="28">
         <f>(PI()/4)*(E7^2-E11^2)</f>
         <v>0.23910975845737278</v>
@@ -12126,17 +12112,17 @@
       <c r="F12" s="24" t="s">
         <v>251</v>
       </c>
-      <c r="I12" s="43" t="s">
+      <c r="I12" s="50" t="s">
         <v>223</v>
       </c>
-      <c r="J12" s="44"/>
-      <c r="K12" s="45"/>
+      <c r="J12" s="51"/>
+      <c r="K12" s="52"/>
     </row>
     <row r="13" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C13" s="46" t="s">
+      <c r="C13" s="53" t="s">
         <v>247</v>
       </c>
-      <c r="D13" s="46"/>
+      <c r="D13" s="53"/>
       <c r="E13" s="31">
         <f>E12*E6*(E9*12)</f>
         <v>127.92780285649083</v>
@@ -12167,12 +12153,12 @@
       </c>
     </row>
     <row r="15" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C15" s="38" t="s">
+      <c r="C15" s="45" t="s">
         <v>253</v>
       </c>
-      <c r="D15" s="38"/>
-      <c r="E15" s="38"/>
-      <c r="F15" s="38"/>
+      <c r="D15" s="45"/>
+      <c r="E15" s="45"/>
+      <c r="F15" s="45"/>
       <c r="I15" s="24" t="s">
         <v>219</v>
       </c>
@@ -12184,10 +12170,10 @@
       </c>
     </row>
     <row r="16" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C16" s="46" t="s">
+      <c r="C16" s="53" t="s">
         <v>8</v>
       </c>
-      <c r="D16" s="46"/>
+      <c r="D16" s="53"/>
       <c r="E16" s="27" t="s">
         <v>5</v>
       </c>
@@ -12205,12 +12191,12 @@
       </c>
     </row>
     <row r="17" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C17" s="34" t="s">
+      <c r="C17" s="41" t="s">
         <v>223</v>
       </c>
-      <c r="D17" s="34"/>
-      <c r="E17" s="34"/>
-      <c r="F17" s="34"/>
+      <c r="D17" s="41"/>
+      <c r="E17" s="41"/>
+      <c r="F17" s="41"/>
       <c r="I17" s="24" t="s">
         <v>220</v>
       </c>
@@ -12222,10 +12208,10 @@
       </c>
     </row>
     <row r="18" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C18" s="41" t="s">
+      <c r="C18" s="48" t="s">
         <v>259</v>
       </c>
-      <c r="D18" s="42"/>
+      <c r="D18" s="49"/>
       <c r="E18" s="24">
         <v>0.28360000000000002</v>
       </c>
@@ -12243,27 +12229,27 @@
       </c>
     </row>
     <row r="19" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C19" s="41" t="s">
+      <c r="C19" s="48" t="s">
         <v>284</v>
       </c>
-      <c r="D19" s="42"/>
+      <c r="D19" s="49"/>
       <c r="E19" s="24">
         <v>15</v>
       </c>
       <c r="F19" s="24" t="s">
         <v>244</v>
       </c>
-      <c r="I19" s="34" t="s">
+      <c r="I19" s="41" t="s">
         <v>234</v>
       </c>
-      <c r="J19" s="34"/>
-      <c r="K19" s="34"/>
+      <c r="J19" s="41"/>
+      <c r="K19" s="41"/>
     </row>
     <row r="20" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C20" s="41" t="s">
+      <c r="C20" s="48" t="s">
         <v>260</v>
       </c>
-      <c r="D20" s="42"/>
+      <c r="D20" s="49"/>
       <c r="E20" s="24">
         <v>1</v>
       </c>
@@ -12282,10 +12268,10 @@
       </c>
     </row>
     <row r="21" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C21" s="41" t="s">
+      <c r="C21" s="48" t="s">
         <v>261</v>
       </c>
-      <c r="D21" s="42"/>
+      <c r="D21" s="49"/>
       <c r="E21" s="24">
         <v>8.3000000000000004E-2</v>
       </c>
@@ -12304,10 +12290,10 @@
       </c>
     </row>
     <row r="22" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C22" s="41" t="s">
+      <c r="C22" s="48" t="s">
         <v>288</v>
       </c>
-      <c r="D22" s="42"/>
+      <c r="D22" s="49"/>
       <c r="E22" s="24">
         <v>20</v>
       </c>
@@ -12326,10 +12312,10 @@
       </c>
     </row>
     <row r="23" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C23" s="41" t="s">
+      <c r="C23" s="48" t="s">
         <v>262</v>
       </c>
-      <c r="D23" s="42"/>
+      <c r="D23" s="49"/>
       <c r="E23" s="24">
         <v>0.15</v>
       </c>
@@ -12348,10 +12334,10 @@
       </c>
     </row>
     <row r="24" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C24" s="41" t="s">
+      <c r="C24" s="48" t="s">
         <v>263</v>
       </c>
-      <c r="D24" s="42"/>
+      <c r="D24" s="49"/>
       <c r="E24" s="24">
         <v>64</v>
       </c>
@@ -12370,10 +12356,10 @@
       </c>
     </row>
     <row r="25" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C25" s="41" t="s">
+      <c r="C25" s="48" t="s">
         <v>264</v>
       </c>
-      <c r="D25" s="42"/>
+      <c r="D25" s="49"/>
       <c r="E25" s="24">
         <v>0.15</v>
       </c>
@@ -12392,199 +12378,197 @@
       </c>
     </row>
     <row r="26" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C26" s="41" t="s">
+      <c r="C26" s="48" t="s">
         <v>265</v>
       </c>
-      <c r="D26" s="42"/>
+      <c r="D26" s="49"/>
       <c r="E26" s="24">
         <v>64</v>
       </c>
       <c r="F26" s="24" t="s">
         <v>285</v>
       </c>
-      <c r="I26" s="43" t="s">
+      <c r="I26" s="50" t="s">
         <v>236</v>
       </c>
-      <c r="J26" s="44"/>
-      <c r="K26" s="45"/>
+      <c r="J26" s="51"/>
+      <c r="K26" s="52"/>
     </row>
     <row r="27" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C27" s="41" t="s">
+      <c r="C27" s="48" t="s">
         <v>254</v>
       </c>
-      <c r="D27" s="42"/>
+      <c r="D27" s="49"/>
       <c r="E27" s="24">
         <v>2.2000000000000002</v>
       </c>
       <c r="F27" s="24" t="s">
         <v>252</v>
       </c>
-      <c r="I27" s="64" t="s">
+      <c r="I27" s="24" t="s">
         <v>237</v>
       </c>
-      <c r="J27" s="65">
+      <c r="J27" s="25">
         <f>J22*(J18/2000)*J17</f>
         <v>965.30309524589188</v>
       </c>
-      <c r="K27" s="64" t="s">
+      <c r="K27" s="24" t="s">
         <v>239</v>
       </c>
     </row>
     <row r="28" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C28" s="41" t="s">
+      <c r="C28" s="48" t="s">
         <v>255</v>
       </c>
-      <c r="D28" s="42"/>
+      <c r="D28" s="49"/>
       <c r="E28" s="24">
         <v>0.15</v>
       </c>
       <c r="F28" s="24" t="s">
         <v>252</v>
       </c>
-      <c r="I28" s="64" t="s">
+      <c r="I28" s="24" t="s">
         <v>238</v>
       </c>
-      <c r="J28" s="65">
+      <c r="J28" s="25">
         <f>J23*(J18/2000)*J17</f>
         <v>318.94517474498764</v>
       </c>
-      <c r="K28" s="64" t="s">
+      <c r="K28" s="24" t="s">
         <v>239</v>
       </c>
     </row>
     <row r="29" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C29" s="41" t="s">
+      <c r="C29" s="48" t="s">
         <v>256</v>
       </c>
-      <c r="D29" s="42"/>
+      <c r="D29" s="49"/>
       <c r="E29" s="24">
         <v>1.5</v>
       </c>
       <c r="F29" s="24" t="s">
         <v>252</v>
       </c>
-      <c r="I29" s="27" t="s">
-        <v>344</v>
-      </c>
-      <c r="J29" s="31">
-        <f>J27/2</f>
-        <v>482.65154762294594</v>
-      </c>
-      <c r="K29" s="27" t="s">
-        <v>239</v>
-      </c>
     </row>
     <row r="30" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C30" s="41" t="s">
+      <c r="C30" s="48" t="s">
         <v>286</v>
       </c>
-      <c r="D30" s="42"/>
+      <c r="D30" s="49"/>
       <c r="E30" s="24">
         <v>1</v>
       </c>
       <c r="F30" s="24" t="s">
         <v>252</v>
       </c>
-      <c r="I30" s="27" t="s">
-        <v>345</v>
-      </c>
-      <c r="J30" s="31">
-        <f>J28/2</f>
-        <v>159.47258737249382</v>
-      </c>
-      <c r="K30" s="27" t="s">
-        <v>239</v>
-      </c>
+      <c r="I30" s="45" t="s">
+        <v>297</v>
+      </c>
+      <c r="J30" s="45"/>
+      <c r="K30" s="45"/>
     </row>
     <row r="31" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C31" s="41" t="s">
+      <c r="C31" s="48" t="s">
         <v>257</v>
       </c>
-      <c r="D31" s="42"/>
+      <c r="D31" s="49"/>
       <c r="E31" s="24">
         <v>13</v>
       </c>
       <c r="F31" s="24" t="s">
         <v>252</v>
       </c>
+      <c r="I31" s="27" t="s">
+        <v>8</v>
+      </c>
+      <c r="J31" s="27" t="s">
+        <v>5</v>
+      </c>
+      <c r="K31" s="27" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="32" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C32" s="41" t="s">
+      <c r="C32" s="48" t="s">
         <v>258</v>
       </c>
-      <c r="D32" s="42"/>
+      <c r="D32" s="49"/>
       <c r="E32" s="24">
         <v>15</v>
       </c>
       <c r="F32" s="24" t="s">
         <v>252</v>
       </c>
-      <c r="I32" s="59" t="s">
-        <v>297</v>
-      </c>
-      <c r="J32" s="59"/>
-      <c r="K32" s="59"/>
+      <c r="I32" s="41" t="s">
+        <v>298</v>
+      </c>
+      <c r="J32" s="41"/>
+      <c r="K32" s="41"/>
     </row>
     <row r="33" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C33" s="41" t="s">
+      <c r="C33" s="48" t="s">
         <v>266</v>
       </c>
-      <c r="D33" s="42"/>
+      <c r="D33" s="49"/>
       <c r="E33" s="24">
         <v>2.5</v>
       </c>
       <c r="F33" s="24" t="s">
         <v>252</v>
       </c>
-      <c r="I33" s="27" t="s">
-        <v>8</v>
-      </c>
-      <c r="J33" s="27" t="s">
-        <v>5</v>
-      </c>
-      <c r="K33" s="27" t="s">
-        <v>6</v>
+      <c r="I33" s="24" t="s">
+        <v>305</v>
+      </c>
+      <c r="J33" s="24">
+        <v>0.45</v>
+      </c>
+      <c r="K33" s="24" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="34" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C34" s="41" t="s">
+      <c r="C34" s="48" t="s">
         <v>270</v>
       </c>
-      <c r="D34" s="42"/>
+      <c r="D34" s="49"/>
       <c r="E34" s="24">
         <v>2</v>
       </c>
       <c r="F34" s="24" t="s">
         <v>252</v>
       </c>
-      <c r="I34" s="60" t="s">
-        <v>298</v>
-      </c>
-      <c r="J34" s="60"/>
-      <c r="K34" s="60"/>
+      <c r="I34" s="24" t="s">
+        <v>306</v>
+      </c>
+      <c r="J34" s="24">
+        <v>0.45</v>
+      </c>
+      <c r="K34" s="24" t="s">
+        <v>95</v>
+      </c>
     </row>
     <row r="35" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C35" s="34" t="s">
+      <c r="C35" s="41" t="s">
         <v>249</v>
       </c>
-      <c r="D35" s="34"/>
-      <c r="E35" s="34"/>
-      <c r="F35" s="34"/>
+      <c r="D35" s="41"/>
+      <c r="E35" s="41"/>
+      <c r="F35" s="41"/>
       <c r="I35" s="24" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="J35" s="24">
-        <v>0.45</v>
+        <v>96</v>
       </c>
       <c r="K35" s="24" t="s">
-        <v>95</v>
+        <v>56</v>
       </c>
     </row>
     <row r="36" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C36" s="41" t="s">
+      <c r="C36" s="48" t="s">
         <v>267</v>
       </c>
-      <c r="D36" s="42"/>
+      <c r="D36" s="49"/>
       <c r="E36" s="24">
         <f>E20-2*E21</f>
         <v>0.83399999999999996</v>
@@ -12593,20 +12577,20 @@
         <v>252</v>
       </c>
       <c r="I36" s="24" t="s">
-        <v>304</v>
+        <v>320</v>
       </c>
       <c r="J36" s="24">
-        <v>0.45</v>
+        <v>1.23</v>
       </c>
       <c r="K36" s="24" t="s">
-        <v>95</v>
+        <v>322</v>
       </c>
     </row>
     <row r="37" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C37" s="41" t="s">
+      <c r="C37" s="48" t="s">
         <v>268</v>
       </c>
-      <c r="D37" s="42"/>
+      <c r="D37" s="49"/>
       <c r="E37" s="28">
         <f>(PI()/4)*(E20^2-E36^2)</f>
         <v>0.23910975845737278</v>
@@ -12615,20 +12599,20 @@
         <v>252</v>
       </c>
       <c r="I37" s="24" t="s">
-        <v>300</v>
+        <v>321</v>
       </c>
       <c r="J37" s="24">
-        <v>93</v>
+        <v>1.23</v>
       </c>
       <c r="K37" s="24" t="s">
-        <v>56</v>
+        <v>322</v>
       </c>
     </row>
     <row r="38" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C38" s="41" t="s">
+      <c r="C38" s="48" t="s">
         <v>287</v>
       </c>
-      <c r="D38" s="42"/>
+      <c r="D38" s="49"/>
       <c r="E38" s="28">
         <f>E37*E18*((E19*E22))</f>
         <v>20.343458249553276</v>
@@ -12640,17 +12624,17 @@
         <v>318</v>
       </c>
       <c r="J38" s="24">
-        <v>1.75</v>
+        <v>0.75</v>
       </c>
       <c r="K38" s="24" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
     </row>
     <row r="39" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C39" s="39" t="s">
+      <c r="C39" s="46" t="s">
         <v>269</v>
       </c>
-      <c r="D39" s="40"/>
+      <c r="D39" s="47"/>
       <c r="E39" s="31">
         <f>E38 + E23*E24 + E25*E26 + E30*4 + E29*4 + E28*8 + E27*4 + E31*4 + E32*4 + E33 + E34</f>
         <v>176.04345824955328</v>
@@ -12662,45 +12646,45 @@
         <v>319</v>
       </c>
       <c r="J39" s="24">
-        <v>1.23</v>
+        <v>0.75</v>
       </c>
       <c r="K39" s="24" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
     </row>
     <row r="40" spans="3:11" x14ac:dyDescent="0.25">
       <c r="I40" s="24" t="s">
-        <v>316</v>
+        <v>301</v>
       </c>
       <c r="J40" s="24">
-        <v>0.81</v>
+        <v>3</v>
       </c>
       <c r="K40" s="24" t="s">
-        <v>320</v>
+        <v>95</v>
       </c>
     </row>
     <row r="41" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C41" s="38" t="s">
+      <c r="C41" s="45" t="s">
         <v>271</v>
       </c>
-      <c r="D41" s="38"/>
-      <c r="E41" s="38"/>
-      <c r="F41" s="38"/>
+      <c r="D41" s="45"/>
+      <c r="E41" s="45"/>
+      <c r="F41" s="45"/>
       <c r="I41" s="24" t="s">
-        <v>317</v>
+        <v>299</v>
       </c>
       <c r="J41" s="24">
-        <v>0.81</v>
+        <v>0.6</v>
       </c>
       <c r="K41" s="24" t="s">
-        <v>320</v>
+        <v>95</v>
       </c>
     </row>
     <row r="42" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C42" s="46" t="s">
+      <c r="C42" s="53" t="s">
         <v>8</v>
       </c>
-      <c r="D42" s="46"/>
+      <c r="D42" s="53"/>
       <c r="E42" s="27" t="s">
         <v>5</v>
       </c>
@@ -12708,37 +12692,33 @@
         <v>6</v>
       </c>
       <c r="I42" s="24" t="s">
-        <v>301</v>
+        <v>310</v>
       </c>
       <c r="J42" s="24">
-        <v>5</v>
+        <v>2000</v>
       </c>
       <c r="K42" s="24" t="s">
-        <v>95</v>
+        <v>226</v>
       </c>
     </row>
     <row r="43" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C43" s="34" t="s">
+      <c r="C43" s="41" t="s">
         <v>223</v>
       </c>
-      <c r="D43" s="34"/>
-      <c r="E43" s="34"/>
-      <c r="F43" s="34"/>
-      <c r="I43" s="24" t="s">
-        <v>299</v>
-      </c>
-      <c r="J43" s="24">
-        <v>0.6</v>
-      </c>
-      <c r="K43" s="24" t="s">
-        <v>95</v>
-      </c>
+      <c r="D43" s="41"/>
+      <c r="E43" s="41"/>
+      <c r="F43" s="41"/>
+      <c r="I43" s="50" t="s">
+        <v>249</v>
+      </c>
+      <c r="J43" s="51"/>
+      <c r="K43" s="52"/>
     </row>
     <row r="44" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C44" s="41" t="s">
+      <c r="C44" s="48" t="s">
         <v>272</v>
       </c>
-      <c r="D44" s="42"/>
+      <c r="D44" s="49"/>
       <c r="E44" s="24">
         <v>136</v>
       </c>
@@ -12746,81 +12726,87 @@
         <v>252</v>
       </c>
       <c r="I44" s="24" t="s">
-        <v>308</v>
-      </c>
-      <c r="J44" s="24">
-        <v>2000</v>
+        <v>302</v>
+      </c>
+      <c r="J44" s="25">
+        <f>2*J33*(J50*6894.76)*(J36*0.0254^2)*(J35/1000)</f>
+        <v>482.651547622946</v>
       </c>
       <c r="K44" s="24" t="s">
-        <v>226</v>
+        <v>239</v>
       </c>
     </row>
     <row r="45" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C45" s="41" t="s">
+      <c r="C45" s="48" t="s">
         <v>273</v>
       </c>
-      <c r="D45" s="42"/>
+      <c r="D45" s="49"/>
       <c r="E45" s="24">
         <v>50</v>
       </c>
       <c r="F45" s="24" t="s">
         <v>252</v>
       </c>
-      <c r="I45" s="61" t="s">
-        <v>249</v>
-      </c>
-      <c r="J45" s="62"/>
-      <c r="K45" s="63"/>
+      <c r="I45" s="24" t="s">
+        <v>303</v>
+      </c>
+      <c r="J45" s="25">
+        <f>2*J34*(J51*6894.76)*(J37*0.0254^2)*(J35/1000)</f>
+        <v>159.47258737249385</v>
+      </c>
+      <c r="K45" s="24" t="s">
+        <v>239</v>
+      </c>
     </row>
     <row r="46" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C46" s="41" t="s">
+      <c r="C46" s="48" t="s">
         <v>274</v>
       </c>
-      <c r="D46" s="42"/>
+      <c r="D46" s="49"/>
       <c r="E46" s="24">
         <v>11</v>
       </c>
       <c r="F46" s="24" t="s">
         <v>252</v>
       </c>
-      <c r="I46" s="27" t="s">
-        <v>346</v>
-      </c>
-      <c r="J46" s="31">
-        <f>2*J35*(J52*6894.76)*J48*(J37/1000)</f>
-        <v>482.65154762294588</v>
-      </c>
-      <c r="K46" s="27" t="s">
-        <v>239</v>
+      <c r="I46" s="24" t="s">
+        <v>304</v>
+      </c>
+      <c r="J46" s="29">
+        <f>J36*0.0254^2</f>
+        <v>7.9354679999999996E-4</v>
+      </c>
+      <c r="K46" s="24" t="s">
+        <v>323</v>
       </c>
     </row>
     <row r="47" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C47" s="41" t="s">
+      <c r="C47" s="48" t="s">
         <v>289</v>
       </c>
-      <c r="D47" s="42"/>
+      <c r="D47" s="49"/>
       <c r="E47" s="24">
         <v>3</v>
       </c>
       <c r="F47" s="24" t="s">
         <v>285</v>
       </c>
-      <c r="I47" s="27" t="s">
-        <v>347</v>
-      </c>
-      <c r="J47" s="31">
-        <f>2*J36*(J53*6894.76)*J49*(J37/1000)</f>
-        <v>159.47258737249382</v>
-      </c>
-      <c r="K47" s="27" t="s">
-        <v>239</v>
+      <c r="I47" s="24" t="s">
+        <v>307</v>
+      </c>
+      <c r="J47" s="29">
+        <f>J37*0.0254^2</f>
+        <v>7.9354679999999996E-4</v>
+      </c>
+      <c r="K47" s="24" t="s">
+        <v>323</v>
       </c>
     </row>
     <row r="48" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C48" s="41" t="s">
+      <c r="C48" s="48" t="s">
         <v>270</v>
       </c>
-      <c r="D48" s="42"/>
+      <c r="D48" s="49"/>
       <c r="E48" s="24">
         <v>5</v>
       </c>
@@ -12828,39 +12814,39 @@
         <v>252</v>
       </c>
       <c r="I48" s="24" t="s">
-        <v>302</v>
+        <v>308</v>
       </c>
       <c r="J48" s="29">
         <f>PI()/4*(J38*0.0254)^2</f>
-        <v>1.5517916547360866E-3</v>
+        <v>2.8502295699234242E-4</v>
       </c>
       <c r="K48" s="24" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
     </row>
     <row r="49" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C49" s="34" t="s">
+      <c r="C49" s="41" t="s">
         <v>275</v>
       </c>
-      <c r="D49" s="34"/>
-      <c r="E49" s="34"/>
-      <c r="F49" s="34"/>
+      <c r="D49" s="41"/>
+      <c r="E49" s="41"/>
+      <c r="F49" s="41"/>
       <c r="I49" s="24" t="s">
-        <v>305</v>
+        <v>309</v>
       </c>
       <c r="J49" s="29">
         <f>PI()/4*(J39*0.0254)^2</f>
-        <v>7.6659774512660424E-4</v>
+        <v>2.8502295699234242E-4</v>
       </c>
       <c r="K49" s="24" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
     </row>
     <row r="50" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C50" s="39" t="s">
+      <c r="C50" s="46" t="s">
         <v>276</v>
       </c>
-      <c r="D50" s="40"/>
+      <c r="D50" s="47"/>
       <c r="E50" s="27">
         <f>E44+E45+(E46*E47)+E48</f>
         <v>224</v>
@@ -12869,179 +12855,162 @@
         <v>252</v>
       </c>
       <c r="I50" s="24" t="s">
-        <v>306</v>
-      </c>
-      <c r="J50" s="29">
-        <f>PI()/4*(J40*0.0254)^2</f>
-        <v>3.3245077703586835E-4</v>
+        <v>311</v>
+      </c>
+      <c r="J50" s="25">
+        <f>(J27/2)/(2*J33*(J35/1000)*J46)/6894.76</f>
+        <v>1021.0059254416738</v>
       </c>
       <c r="K50" s="24" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
     </row>
     <row r="51" spans="3:11" x14ac:dyDescent="0.25">
       <c r="I51" s="24" t="s">
-        <v>307</v>
-      </c>
-      <c r="J51" s="29">
-        <f>PI()/4*(J41*0.0254)^2</f>
-        <v>3.3245077703586835E-4</v>
+        <v>312</v>
+      </c>
+      <c r="J51" s="25">
+        <f>(J28/2)/(2*J34*(J35/1000)*J47)/6894.76</f>
+        <v>337.34991103774598</v>
       </c>
       <c r="K51" s="24" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
     </row>
     <row r="52" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C52" s="38" t="s">
+      <c r="C52" s="45" t="s">
         <v>277</v>
       </c>
-      <c r="D52" s="38"/>
-      <c r="E52" s="38"/>
-      <c r="F52" s="38"/>
-      <c r="I52" s="27" t="s">
-        <v>309</v>
-      </c>
-      <c r="J52" s="31">
-        <f>(J27/2)/(2*J35*(J37/1000)*J48)/6894.76</f>
-        <v>538.95893941439783</v>
-      </c>
-      <c r="K52" s="27" t="s">
-        <v>322</v>
+      <c r="D52" s="45"/>
+      <c r="E52" s="45"/>
+      <c r="F52" s="45"/>
+      <c r="I52" s="24" t="s">
+        <v>316</v>
+      </c>
+      <c r="J52" s="25">
+        <f>J42*J40*J41/J48/6894.76</f>
+        <v>1831.9073535403561</v>
+      </c>
+      <c r="K52" s="24" t="s">
+        <v>324</v>
       </c>
     </row>
     <row r="53" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C53" s="46" t="s">
+      <c r="C53" s="53" t="s">
         <v>8</v>
       </c>
-      <c r="D53" s="46"/>
+      <c r="D53" s="53"/>
       <c r="E53" s="27" t="s">
         <v>5</v>
       </c>
       <c r="F53" s="27" t="s">
         <v>6</v>
       </c>
-      <c r="I53" s="27" t="s">
-        <v>310</v>
-      </c>
-      <c r="J53" s="31">
-        <f>(J28/2)/(2*J36*(J37/1000)*J49)/6894.76</f>
-        <v>360.47395511871792</v>
-      </c>
-      <c r="K53" s="27" t="s">
-        <v>322</v>
+      <c r="I53" s="24" t="s">
+        <v>317</v>
+      </c>
+      <c r="J53" s="25">
+        <f>J42*J40*(1-J41)/J49/6894.76</f>
+        <v>1221.271569026904</v>
+      </c>
+      <c r="K53" s="24" t="s">
+        <v>324</v>
       </c>
     </row>
     <row r="54" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C54" s="43" t="s">
+      <c r="C54" s="50" t="s">
         <v>223</v>
       </c>
-      <c r="D54" s="44"/>
-      <c r="E54" s="44"/>
-      <c r="F54" s="45"/>
-      <c r="I54" s="27" t="s">
-        <v>314</v>
-      </c>
-      <c r="J54" s="31">
-        <f>J44*J42*J43/J50/6894.76</f>
-        <v>2617.6088156440837</v>
-      </c>
-      <c r="K54" s="27" t="s">
-        <v>322</v>
+      <c r="D54" s="51"/>
+      <c r="E54" s="51"/>
+      <c r="F54" s="52"/>
+      <c r="I54" s="24" t="s">
+        <v>313</v>
+      </c>
+      <c r="J54" s="25">
+        <f>J50*6894.76*J48/(J40*J41)</f>
+        <v>1114.691661091344</v>
+      </c>
+      <c r="K54" s="24" t="s">
+        <v>226</v>
       </c>
     </row>
     <row r="55" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C55" s="41" t="s">
+      <c r="C55" s="48" t="s">
         <v>278</v>
       </c>
-      <c r="D55" s="42"/>
+      <c r="D55" s="49"/>
       <c r="E55" s="24">
         <v>175</v>
       </c>
       <c r="F55" s="24" t="s">
         <v>252</v>
       </c>
-      <c r="I55" s="27" t="s">
-        <v>315</v>
-      </c>
-      <c r="J55" s="31">
-        <f>J44*J42*(1-J43)/J51/6894.76</f>
-        <v>1745.0725437627223</v>
-      </c>
-      <c r="K55" s="27" t="s">
-        <v>322</v>
+      <c r="I55" s="24" t="s">
+        <v>314</v>
+      </c>
+      <c r="J55" s="25">
+        <f>J51*6894.76*J49/(J40*(1-J41))</f>
+        <v>552.45683203211331</v>
+      </c>
+      <c r="K55" s="24" t="s">
+        <v>226</v>
       </c>
     </row>
     <row r="56" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C56" s="41" t="s">
+      <c r="C56" s="48" t="s">
         <v>279</v>
       </c>
-      <c r="D56" s="42"/>
+      <c r="D56" s="49"/>
       <c r="E56" s="24">
         <v>5</v>
       </c>
       <c r="F56" s="24" t="s">
         <v>252</v>
       </c>
-      <c r="I56" s="27" t="s">
-        <v>311</v>
-      </c>
-      <c r="J56" s="31">
-        <f>J52*6894.76*J50/(J42*J43)</f>
-        <v>411.79486880799089</v>
-      </c>
-      <c r="K56" s="27" t="s">
+      <c r="I56" s="24" t="s">
+        <v>315</v>
+      </c>
+      <c r="J56" s="25">
+        <f>MAX(J54,J55)</f>
+        <v>1114.691661091344</v>
+      </c>
+      <c r="K56" s="24" t="s">
         <v>226</v>
       </c>
     </row>
     <row r="57" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C57" s="41" t="s">
+      <c r="C57" s="48" t="s">
         <v>280</v>
       </c>
-      <c r="D57" s="42"/>
+      <c r="D57" s="49"/>
       <c r="E57" s="24">
         <v>1</v>
       </c>
       <c r="F57" s="24" t="s">
         <v>252</v>
       </c>
-      <c r="I57" s="27" t="s">
-        <v>312</v>
-      </c>
-      <c r="J57" s="31">
-        <f>J53*6894.76*J51/(J42*(1-J43))</f>
-        <v>413.13348995963759</v>
-      </c>
-      <c r="K57" s="27" t="s">
-        <v>226</v>
+      <c r="J57" t="s">
+        <v>325</v>
       </c>
     </row>
     <row r="58" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C58" s="41" t="s">
+      <c r="C58" s="48" t="s">
         <v>281</v>
       </c>
-      <c r="D58" s="42"/>
+      <c r="D58" s="49"/>
       <c r="E58" s="24">
         <v>3</v>
       </c>
       <c r="F58" s="24" t="s">
         <v>252</v>
       </c>
-      <c r="I58" s="27" t="s">
-        <v>313</v>
-      </c>
-      <c r="J58" s="31">
-        <f>MAX(J56,J57)</f>
-        <v>413.13348995963759</v>
-      </c>
-      <c r="K58" s="27" t="s">
-        <v>226</v>
-      </c>
     </row>
     <row r="59" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C59" s="41" t="s">
+      <c r="C59" s="48" t="s">
         <v>282</v>
       </c>
-      <c r="D59" s="42"/>
+      <c r="D59" s="49"/>
       <c r="E59" s="24">
         <v>1</v>
       </c>
@@ -13050,10 +13019,10 @@
       </c>
     </row>
     <row r="60" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C60" s="41" t="s">
+      <c r="C60" s="48" t="s">
         <v>270</v>
       </c>
-      <c r="D60" s="42"/>
+      <c r="D60" s="49"/>
       <c r="E60" s="24">
         <v>0.5</v>
       </c>
@@ -13062,18 +13031,18 @@
       </c>
     </row>
     <row r="61" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C61" s="34" t="s">
+      <c r="C61" s="41" t="s">
         <v>275</v>
       </c>
-      <c r="D61" s="34"/>
-      <c r="E61" s="34"/>
-      <c r="F61" s="34"/>
+      <c r="D61" s="41"/>
+      <c r="E61" s="41"/>
+      <c r="F61" s="41"/>
     </row>
     <row r="62" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C62" s="39" t="s">
+      <c r="C62" s="46" t="s">
         <v>276</v>
       </c>
-      <c r="D62" s="40"/>
+      <c r="D62" s="47"/>
       <c r="E62" s="31">
         <f>SUM(E55:E60)</f>
         <v>185.5</v>
@@ -13083,7 +13052,7 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="62">
+  <mergeCells count="65">
     <mergeCell ref="I3:K3"/>
     <mergeCell ref="I12:K12"/>
     <mergeCell ref="C3:F3"/>
@@ -13135,11 +13104,14 @@
     <mergeCell ref="C60:D60"/>
     <mergeCell ref="I19:K19"/>
     <mergeCell ref="I10:K10"/>
+    <mergeCell ref="I30:K30"/>
     <mergeCell ref="C62:D62"/>
     <mergeCell ref="C30:D30"/>
     <mergeCell ref="C38:D38"/>
     <mergeCell ref="C46:D46"/>
     <mergeCell ref="I26:K26"/>
+    <mergeCell ref="I32:K32"/>
+    <mergeCell ref="I43:K43"/>
     <mergeCell ref="C18:D18"/>
     <mergeCell ref="C36:D36"/>
     <mergeCell ref="C37:D37"/>

</xml_diff>